<commit_message>
Atualizando cadastro de item novo 12/05
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodosLibanes.xlsx
+++ b/data/ProdutosFomatodosLibanes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\listaProdutosToufic\lista-de-produtos-toufic\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F08226-FF50-41F9-B2FF-B1536D04EF87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D3414BB-1C1A-498C-9C7E-4FB6B7E96079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="570" yWindow="780" windowWidth="27300" windowHeight="13920" firstSheet="8" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="promoçoes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3568" uniqueCount="1102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3572" uniqueCount="1105">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -3343,6 +3343,15 @@
   </si>
   <si>
     <t>BALA GELATINA COBRINHA CITRICA</t>
+  </si>
+  <si>
+    <t>gota-chocolate-branco</t>
+  </si>
+  <si>
+    <t>GOTA CHOCOLATE BRANCO</t>
+  </si>
+  <si>
+    <t>500G</t>
   </si>
 </sst>
 </file>
@@ -9898,7 +9907,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H122"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -12511,54 +12520,54 @@
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>1024</v>
+        <v>1102</v>
       </c>
       <c r="B101" t="s">
-        <v>1025</v>
+        <v>1103</v>
       </c>
       <c r="C101">
-        <v>4412</v>
+        <v>4635</v>
       </c>
       <c r="D101">
-        <v>2.5</v>
+        <v>10</v>
       </c>
       <c r="E101" t="s">
-        <v>10</v>
+        <v>1104</v>
       </c>
       <c r="F101" t="s">
         <v>988</v>
       </c>
       <c r="G101">
-        <v>71.5</v>
+        <v>167</v>
       </c>
       <c r="H101">
-        <v>73.5</v>
+        <v>172</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="B102" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
       <c r="C102">
-        <v>4413</v>
+        <v>4412</v>
       </c>
       <c r="D102">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="E102" t="s">
         <v>10</v>
       </c>
       <c r="F102" t="s">
-        <v>11</v>
+        <v>988</v>
       </c>
       <c r="G102">
-        <v>496</v>
+        <v>71.5</v>
       </c>
       <c r="H102">
-        <v>511</v>
+        <v>73.5</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
@@ -12569,10 +12578,10 @@
         <v>1027</v>
       </c>
       <c r="C103">
-        <v>4414</v>
+        <v>4413</v>
       </c>
       <c r="D103">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E103" t="s">
         <v>10</v>
@@ -12581,24 +12590,24 @@
         <v>11</v>
       </c>
       <c r="G103">
-        <v>101</v>
+        <v>496</v>
       </c>
       <c r="H103">
-        <v>104</v>
+        <v>511</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="B104" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
       <c r="C104">
-        <v>4415</v>
+        <v>4414</v>
       </c>
       <c r="D104">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E104" t="s">
         <v>10</v>
@@ -12607,10 +12616,10 @@
         <v>11</v>
       </c>
       <c r="G104">
-        <v>414</v>
+        <v>101</v>
       </c>
       <c r="H104">
-        <v>426.5</v>
+        <v>104</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.25">
@@ -12621,10 +12630,10 @@
         <v>1029</v>
       </c>
       <c r="C105">
-        <v>4416</v>
+        <v>4415</v>
       </c>
       <c r="D105">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E105" t="s">
         <v>10</v>
@@ -12633,73 +12642,73 @@
         <v>11</v>
       </c>
       <c r="G105">
-        <v>85</v>
+        <v>414</v>
       </c>
       <c r="H105">
-        <v>87</v>
+        <v>426.5</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
       <c r="B106" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="C106">
-        <v>4475</v>
+        <v>4416</v>
       </c>
       <c r="D106">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E106" t="s">
-        <v>1032</v>
+        <v>10</v>
       </c>
       <c r="F106" t="s">
         <v>11</v>
       </c>
       <c r="G106">
-        <v>9</v>
+        <v>85</v>
       </c>
       <c r="H106">
-        <v>9.5</v>
+        <v>87</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>1033</v>
+        <v>1030</v>
       </c>
       <c r="B107" t="s">
-        <v>1034</v>
+        <v>1031</v>
       </c>
       <c r="C107">
-        <v>4354</v>
+        <v>4475</v>
       </c>
       <c r="D107">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E107" t="s">
         <v>1032</v>
       </c>
       <c r="F107" t="s">
-        <v>750</v>
+        <v>11</v>
       </c>
       <c r="G107">
-        <v>79.5</v>
+        <v>9</v>
       </c>
       <c r="H107">
-        <v>82</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>1035</v>
+        <v>1033</v>
       </c>
       <c r="B108" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="C108">
-        <v>4445</v>
+        <v>4354</v>
       </c>
       <c r="D108">
         <v>12</v>
@@ -12708,7 +12717,7 @@
         <v>1032</v>
       </c>
       <c r="F108" t="s">
-        <v>25</v>
+        <v>750</v>
       </c>
       <c r="G108">
         <v>79.5</v>
@@ -12719,13 +12728,13 @@
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
       <c r="B109" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="C109">
-        <v>4353</v>
+        <v>4445</v>
       </c>
       <c r="D109">
         <v>12</v>
@@ -12745,13 +12754,13 @@
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="B110" t="s">
-        <v>1040</v>
+        <v>1038</v>
       </c>
       <c r="C110">
-        <v>4350</v>
+        <v>4353</v>
       </c>
       <c r="D110">
         <v>12</v>
@@ -12771,13 +12780,13 @@
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
       <c r="B111" t="s">
-        <v>1042</v>
+        <v>1040</v>
       </c>
       <c r="C111">
-        <v>4352</v>
+        <v>4350</v>
       </c>
       <c r="D111">
         <v>12</v>
@@ -12797,13 +12806,13 @@
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
       <c r="B112" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
       <c r="C112">
-        <v>4349</v>
+        <v>4352</v>
       </c>
       <c r="D112">
         <v>12</v>
@@ -12823,13 +12832,13 @@
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="B113" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
       <c r="C113">
-        <v>4351</v>
+        <v>4349</v>
       </c>
       <c r="D113">
         <v>12</v>
@@ -12849,13 +12858,13 @@
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
       <c r="B114" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
       <c r="C114">
-        <v>4581</v>
+        <v>4351</v>
       </c>
       <c r="D114">
         <v>12</v>
@@ -12875,91 +12884,91 @@
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="B115" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
       <c r="C115">
-        <v>4096</v>
+        <v>4581</v>
       </c>
       <c r="D115">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E115" t="s">
-        <v>10</v>
+        <v>1032</v>
       </c>
       <c r="F115" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G115">
-        <v>79</v>
+        <v>79.5</v>
       </c>
       <c r="H115">
-        <v>81.5</v>
+        <v>82</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="B116" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="C116">
-        <v>4123</v>
+        <v>4096</v>
       </c>
       <c r="D116">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E116" t="s">
-        <v>1016</v>
+        <v>10</v>
       </c>
       <c r="F116" t="s">
         <v>11</v>
       </c>
       <c r="G116">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="H116">
-        <v>62</v>
+        <v>81.5</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="B117" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="C117">
-        <v>4306</v>
+        <v>4123</v>
       </c>
       <c r="D117">
         <v>10</v>
       </c>
       <c r="E117" t="s">
-        <v>1003</v>
+        <v>1016</v>
       </c>
       <c r="F117" t="s">
-        <v>988</v>
+        <v>11</v>
       </c>
       <c r="G117">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="H117">
-        <v>83.5</v>
+        <v>62</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
       <c r="B118" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="C118">
-        <v>4307</v>
+        <v>4306</v>
       </c>
       <c r="D118">
         <v>10</v>
@@ -12979,28 +12988,28 @@
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="B119" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C119">
-        <v>2659</v>
+        <v>4307</v>
       </c>
       <c r="D119">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E119" t="s">
-        <v>1059</v>
+        <v>1003</v>
       </c>
       <c r="F119" t="s">
-        <v>33</v>
+        <v>988</v>
       </c>
       <c r="G119">
-        <v>27.5</v>
+        <v>81</v>
       </c>
       <c r="H119">
-        <v>28.5</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.25">
@@ -13011,47 +13020,73 @@
         <v>1058</v>
       </c>
       <c r="C120">
-        <v>2621</v>
+        <v>2659</v>
       </c>
       <c r="D120">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E120" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="F120" t="s">
         <v>33</v>
       </c>
       <c r="G120">
-        <v>24.5</v>
+        <v>27.5</v>
       </c>
       <c r="H120">
-        <v>25</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>1061</v>
+        <v>1057</v>
       </c>
       <c r="B121" t="s">
-        <v>1062</v>
+        <v>1058</v>
       </c>
       <c r="C121">
-        <v>3656</v>
+        <v>2621</v>
       </c>
       <c r="D121">
         <v>5</v>
       </c>
       <c r="E121" t="s">
-        <v>1003</v>
+        <v>1060</v>
       </c>
       <c r="F121" t="s">
         <v>33</v>
       </c>
       <c r="G121">
+        <v>24.5</v>
+      </c>
+      <c r="H121">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B122" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C122">
+        <v>3656</v>
+      </c>
+      <c r="D122">
+        <v>5</v>
+      </c>
+      <c r="E122" t="s">
+        <v>1003</v>
+      </c>
+      <c r="F122" t="s">
+        <v>33</v>
+      </c>
+      <c r="G122">
         <v>27</v>
       </c>
-      <c r="H121">
+      <c r="H122">
         <v>28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizando preço e produtos novos 21/05
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodosLibanes.xlsx
+++ b/data/ProdutosFomatodosLibanes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\listaProdutosToufic\lista-de-produtos-toufic\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AEAA872-EFFF-4855-BE43-4F5AA6E21133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDA5D795-263B-421C-8C22-3DE2DDAB0DCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" firstSheet="11" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="promoçoes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3580" uniqueCount="1107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3592" uniqueCount="1111">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -3358,6 +3358,18 @@
   </si>
   <si>
     <t>CASTANHA DO PARA LARGE PARATINI</t>
+  </si>
+  <si>
+    <t>ameixa-em-po</t>
+  </si>
+  <si>
+    <t>AMEIXA EM PÓ</t>
+  </si>
+  <si>
+    <t>flocos-de-arroz</t>
+  </si>
+  <si>
+    <t>FLOCOS DE ARROZ</t>
   </si>
 </sst>
 </file>
@@ -5559,7 +5571,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:H113"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -5772,10 +5784,10 @@
         <v>33</v>
       </c>
       <c r="G8">
-        <v>57.5</v>
+        <v>62</v>
       </c>
       <c r="H8">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -5798,10 +5810,10 @@
         <v>33</v>
       </c>
       <c r="G9">
-        <v>65</v>
+        <v>69.5</v>
       </c>
       <c r="H9">
-        <v>67</v>
+        <v>71.5</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5824,10 +5836,10 @@
         <v>33</v>
       </c>
       <c r="G10">
-        <v>141.5</v>
+        <v>153.5</v>
       </c>
       <c r="H10">
-        <v>146</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -6014,28 +6026,28 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>666</v>
+        <v>1107</v>
       </c>
       <c r="B18" t="s">
-        <v>667</v>
+        <v>1108</v>
       </c>
       <c r="C18">
-        <v>2336</v>
+        <v>4639</v>
       </c>
       <c r="D18">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G18">
-        <v>750</v>
+        <v>295</v>
       </c>
       <c r="H18">
-        <v>772.5</v>
+        <v>304</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -6046,48 +6058,48 @@
         <v>667</v>
       </c>
       <c r="C19">
-        <v>2421</v>
+        <v>2336</v>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
       </c>
       <c r="F19" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G19">
-        <v>91</v>
+        <v>750</v>
       </c>
       <c r="H19">
-        <v>94</v>
+        <v>772.5</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="B20" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="C20">
-        <v>2568</v>
+        <v>2421</v>
       </c>
       <c r="D20">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G20">
-        <v>260</v>
+        <v>91</v>
       </c>
       <c r="H20">
-        <v>268</v>
+        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -6098,59 +6110,59 @@
         <v>669</v>
       </c>
       <c r="C21">
-        <v>3009</v>
+        <v>2568</v>
       </c>
       <c r="D21">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
       </c>
       <c r="F21" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G21">
-        <v>78</v>
+        <v>260</v>
       </c>
       <c r="H21">
-        <v>80.5</v>
+        <v>268</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B22" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="C22">
-        <v>2778</v>
+        <v>3009</v>
       </c>
       <c r="D22">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
       </c>
       <c r="F22" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G22">
-        <v>180</v>
+        <v>78</v>
       </c>
       <c r="H22">
-        <v>185.5</v>
+        <v>80.5</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="B23" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="C23">
-        <v>3106</v>
+        <v>2778</v>
       </c>
       <c r="D23">
         <v>5</v>
@@ -6159,39 +6171,39 @@
         <v>10</v>
       </c>
       <c r="F23" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G23">
-        <v>260</v>
+        <v>180</v>
       </c>
       <c r="H23">
-        <v>268</v>
+        <v>185.5</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="B24" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="C24">
-        <v>3489</v>
+        <v>3106</v>
       </c>
       <c r="D24">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
       </c>
       <c r="F24" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G24">
-        <v>700</v>
+        <v>260</v>
       </c>
       <c r="H24">
-        <v>721</v>
+        <v>268</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -6202,22 +6214,22 @@
         <v>675</v>
       </c>
       <c r="C25">
-        <v>2783</v>
+        <v>3489</v>
       </c>
       <c r="D25">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G25">
-        <v>142</v>
+        <v>700</v>
       </c>
       <c r="H25">
-        <v>159.5</v>
+        <v>721</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -6228,10 +6240,10 @@
         <v>675</v>
       </c>
       <c r="C26">
-        <v>3755</v>
+        <v>2783</v>
       </c>
       <c r="D26">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -6240,36 +6252,36 @@
         <v>11</v>
       </c>
       <c r="G26">
-        <v>85</v>
+        <v>142</v>
       </c>
       <c r="H26">
-        <v>88</v>
+        <v>159.5</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="B27" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="C27">
-        <v>3486</v>
+        <v>3755</v>
       </c>
       <c r="D27">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
       </c>
       <c r="F27" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G27">
-        <v>595</v>
+        <v>85</v>
       </c>
       <c r="H27">
-        <v>613</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -6280,10 +6292,10 @@
         <v>677</v>
       </c>
       <c r="C28">
-        <v>4488</v>
+        <v>3487</v>
       </c>
       <c r="D28">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -6292,47 +6304,47 @@
         <v>11</v>
       </c>
       <c r="G28">
-        <v>299.5</v>
+        <v>180</v>
       </c>
       <c r="H28">
-        <v>308.5</v>
+        <v>185.5</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="B29" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="C29">
-        <v>4333</v>
+        <v>3486</v>
       </c>
       <c r="D29">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
       </c>
       <c r="F29" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G29">
-        <v>259.5</v>
+        <v>595</v>
       </c>
       <c r="H29">
-        <v>267</v>
+        <v>613</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="B30" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="C30">
-        <v>4388</v>
+        <v>4488</v>
       </c>
       <c r="D30">
         <v>5</v>
@@ -6344,21 +6356,21 @@
         <v>11</v>
       </c>
       <c r="G30">
-        <v>145</v>
+        <v>299.5</v>
       </c>
       <c r="H30">
-        <v>149.5</v>
+        <v>308.5</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="B31" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
       <c r="C31">
-        <v>4389</v>
+        <v>4333</v>
       </c>
       <c r="D31">
         <v>5</v>
@@ -6370,47 +6382,47 @@
         <v>11</v>
       </c>
       <c r="G31">
-        <v>102</v>
+        <v>259.5</v>
       </c>
       <c r="H31">
-        <v>105</v>
+        <v>267</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
       <c r="B32" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="C32">
-        <v>3488</v>
+        <v>4388</v>
       </c>
       <c r="D32">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
       </c>
       <c r="F32" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G32">
-        <v>220</v>
+        <v>145</v>
       </c>
       <c r="H32">
-        <v>226.5</v>
+        <v>149.5</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B33" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="C33">
-        <v>3400</v>
+        <v>4389</v>
       </c>
       <c r="D33">
         <v>5</v>
@@ -6422,73 +6434,73 @@
         <v>11</v>
       </c>
       <c r="G33">
-        <v>57</v>
+        <v>102</v>
       </c>
       <c r="H33">
-        <v>59</v>
+        <v>105</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>95</v>
+        <v>684</v>
       </c>
       <c r="B34" t="s">
-        <v>96</v>
+        <v>685</v>
       </c>
       <c r="C34">
-        <v>2257</v>
+        <v>3488</v>
       </c>
       <c r="D34">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
       </c>
       <c r="F34" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G34">
-        <v>16</v>
+        <v>220</v>
       </c>
       <c r="H34">
-        <v>16.5</v>
+        <v>226.5</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>95</v>
+        <v>684</v>
       </c>
       <c r="B35" t="s">
-        <v>96</v>
+        <v>685</v>
       </c>
       <c r="C35">
-        <v>565</v>
+        <v>3400</v>
       </c>
       <c r="D35">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E35" t="s">
         <v>10</v>
       </c>
       <c r="F35" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G35">
-        <v>123</v>
+        <v>57</v>
       </c>
       <c r="H35">
-        <v>129</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>686</v>
+        <v>95</v>
       </c>
       <c r="B36" t="s">
-        <v>687</v>
+        <v>96</v>
       </c>
       <c r="C36">
-        <v>4474</v>
+        <v>2257</v>
       </c>
       <c r="D36">
         <v>3</v>
@@ -6500,47 +6512,47 @@
         <v>11</v>
       </c>
       <c r="G36">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="H36">
-        <v>40</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>688</v>
+        <v>95</v>
       </c>
       <c r="B37" t="s">
-        <v>689</v>
+        <v>96</v>
       </c>
       <c r="C37">
-        <v>4473</v>
+        <v>565</v>
       </c>
       <c r="D37">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="E37" t="s">
         <v>10</v>
       </c>
       <c r="F37" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G37">
-        <v>39</v>
+        <v>123</v>
       </c>
       <c r="H37">
-        <v>40</v>
+        <v>129</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>690</v>
+        <v>686</v>
       </c>
       <c r="B38" t="s">
-        <v>691</v>
+        <v>687</v>
       </c>
       <c r="C38">
-        <v>2658</v>
+        <v>4474</v>
       </c>
       <c r="D38">
         <v>3</v>
@@ -6560,13 +6572,13 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="B39" t="s">
-        <v>693</v>
+        <v>689</v>
       </c>
       <c r="C39">
-        <v>2657</v>
+        <v>4473</v>
       </c>
       <c r="D39">
         <v>3</v>
@@ -6586,276 +6598,276 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>694</v>
+        <v>690</v>
       </c>
       <c r="B40" t="s">
-        <v>695</v>
+        <v>691</v>
       </c>
       <c r="C40">
-        <v>3537</v>
+        <v>2658</v>
       </c>
       <c r="D40">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E40" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F40" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G40">
-        <v>162</v>
+        <v>39</v>
       </c>
       <c r="H40">
-        <v>166.5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
       <c r="B41" t="s">
-        <v>697</v>
+        <v>693</v>
       </c>
       <c r="C41">
-        <v>2732</v>
+        <v>2657</v>
       </c>
       <c r="D41">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E41" t="s">
         <v>10</v>
       </c>
       <c r="F41" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G41">
-        <v>189</v>
+        <v>39</v>
       </c>
       <c r="H41">
-        <v>194.5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>696</v>
+        <v>1109</v>
       </c>
       <c r="B42" t="s">
-        <v>697</v>
+        <v>1110</v>
       </c>
       <c r="C42">
-        <v>2733</v>
+        <v>4640</v>
       </c>
       <c r="D42">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E42" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F42" t="s">
         <v>11</v>
       </c>
       <c r="G42">
-        <v>96.5</v>
+        <v>82.5</v>
       </c>
       <c r="H42">
-        <v>99.5</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
       <c r="B43" t="s">
-        <v>699</v>
+        <v>695</v>
       </c>
       <c r="C43">
-        <v>2584</v>
+        <v>3537</v>
       </c>
       <c r="D43">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F43" t="s">
         <v>25</v>
       </c>
       <c r="G43">
-        <v>223</v>
+        <v>162</v>
       </c>
       <c r="H43">
-        <v>130</v>
+        <v>166.5</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="B44" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="C44">
-        <v>2677</v>
+        <v>2732</v>
       </c>
       <c r="D44">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E44" t="s">
         <v>10</v>
       </c>
       <c r="F44" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G44">
-        <v>113.5</v>
+        <v>189</v>
       </c>
       <c r="H44">
-        <v>117</v>
+        <v>194.5</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="B45" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="C45">
-        <v>2495</v>
+        <v>2733</v>
       </c>
       <c r="D45">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E45" t="s">
         <v>10</v>
       </c>
       <c r="F45" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G45">
-        <v>220</v>
+        <v>96.5</v>
       </c>
       <c r="H45">
-        <v>226.5</v>
+        <v>99.5</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="B46" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="C46">
-        <v>2678</v>
+        <v>2584</v>
       </c>
       <c r="D46">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E46" t="s">
         <v>10</v>
       </c>
       <c r="F46" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G46">
-        <v>112</v>
+        <v>223</v>
       </c>
       <c r="H46">
-        <v>115.5</v>
+        <v>130</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="B47" t="s">
-        <v>703</v>
+        <v>699</v>
       </c>
       <c r="C47">
-        <v>4498</v>
+        <v>2677</v>
       </c>
       <c r="D47">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E47" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F47" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="G47">
-        <v>240</v>
+        <v>113.5</v>
       </c>
       <c r="H47">
-        <v>247</v>
+        <v>117</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="B48" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="C48">
-        <v>4253</v>
+        <v>2495</v>
       </c>
       <c r="D48">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E48" t="s">
         <v>10</v>
       </c>
       <c r="F48" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G48">
-        <v>112</v>
+        <v>220</v>
       </c>
       <c r="H48">
-        <v>115.5</v>
+        <v>226.5</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="B49" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="C49">
-        <v>4500</v>
+        <v>2678</v>
       </c>
       <c r="D49">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E49" t="s">
         <v>10</v>
       </c>
       <c r="F49" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="G49">
-        <v>224</v>
+        <v>112</v>
       </c>
       <c r="H49">
-        <v>230</v>
+        <v>115.5</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="B50" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="C50">
-        <v>4249</v>
+        <v>4498</v>
       </c>
       <c r="D50">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E50" t="s">
         <v>30</v>
@@ -6864,10 +6876,10 @@
         <v>33</v>
       </c>
       <c r="G50">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="H50">
-        <v>237</v>
+        <v>247</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -6878,62 +6890,62 @@
         <v>705</v>
       </c>
       <c r="C51">
-        <v>3724</v>
+        <v>4253</v>
       </c>
       <c r="D51">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E51" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F51" t="s">
         <v>33</v>
       </c>
       <c r="G51">
-        <v>224</v>
+        <v>112</v>
       </c>
       <c r="H51">
-        <v>230</v>
+        <v>115.5</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B52" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="C52">
-        <v>3736</v>
+        <v>4500</v>
       </c>
       <c r="D52">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E52" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G52">
-        <v>162</v>
+        <v>224</v>
       </c>
       <c r="H52">
-        <v>166.5</v>
+        <v>230</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
       <c r="B53" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="C53">
-        <v>4499</v>
+        <v>4249</v>
       </c>
       <c r="D53">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E53" t="s">
         <v>30</v>
@@ -6942,125 +6954,125 @@
         <v>33</v>
       </c>
       <c r="G53">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="H53">
-        <v>247</v>
+        <v>237</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>710</v>
+        <v>704</v>
       </c>
       <c r="B54" t="s">
-        <v>711</v>
+        <v>705</v>
       </c>
       <c r="C54">
-        <v>3536</v>
+        <v>3724</v>
       </c>
       <c r="D54">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E54" t="s">
         <v>30</v>
       </c>
       <c r="F54" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G54">
-        <v>162</v>
+        <v>224</v>
       </c>
       <c r="H54">
-        <v>166.5</v>
+        <v>230</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>712</v>
+        <v>706</v>
       </c>
       <c r="B55" t="s">
-        <v>713</v>
+        <v>707</v>
       </c>
       <c r="C55">
-        <v>2494</v>
+        <v>3736</v>
       </c>
       <c r="D55">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E55" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F55" t="s">
         <v>25</v>
       </c>
       <c r="G55">
-        <v>188.5</v>
+        <v>162</v>
       </c>
       <c r="H55">
-        <v>194</v>
+        <v>166.5</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
       <c r="B56" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
       <c r="C56">
-        <v>2679</v>
+        <v>4499</v>
       </c>
       <c r="D56">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E56" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F56" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="G56">
-        <v>96</v>
+        <v>240</v>
       </c>
       <c r="H56">
-        <v>99</v>
+        <v>247</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
       <c r="B57" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
       <c r="C57">
-        <v>4497</v>
+        <v>3536</v>
       </c>
       <c r="D57">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E57" t="s">
         <v>30</v>
       </c>
       <c r="F57" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G57">
-        <v>240</v>
+        <v>162</v>
       </c>
       <c r="H57">
-        <v>247</v>
+        <v>166.5</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
       <c r="B58" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="C58">
-        <v>2493</v>
+        <v>2494</v>
       </c>
       <c r="D58">
         <v>10</v>
@@ -7072,232 +7084,232 @@
         <v>25</v>
       </c>
       <c r="G58">
-        <v>180</v>
+        <v>188.5</v>
       </c>
       <c r="H58">
-        <v>185.5</v>
+        <v>194</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>718</v>
+        <v>712</v>
       </c>
       <c r="B59" t="s">
-        <v>719</v>
+        <v>713</v>
       </c>
       <c r="C59">
-        <v>3535</v>
+        <v>2679</v>
       </c>
       <c r="D59">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E59" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F59" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G59">
-        <v>162</v>
+        <v>96</v>
       </c>
       <c r="H59">
-        <v>166.5</v>
+        <v>99</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="B60" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="C60">
-        <v>2498</v>
+        <v>4497</v>
       </c>
       <c r="D60">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E60" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F60" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="G60">
-        <v>92</v>
+        <v>240</v>
       </c>
       <c r="H60">
-        <v>94</v>
+        <v>247</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="B61" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
       <c r="C61">
-        <v>2806</v>
+        <v>2493</v>
       </c>
       <c r="D61">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E61" t="s">
         <v>10</v>
       </c>
       <c r="F61" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G61">
-        <v>472.5</v>
+        <v>180</v>
       </c>
       <c r="H61">
-        <v>487</v>
+        <v>185.5</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="B62" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="C62">
-        <v>2807</v>
+        <v>3535</v>
       </c>
       <c r="D62">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E62" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F62" t="s">
         <v>25</v>
       </c>
       <c r="G62">
-        <v>159.5</v>
+        <v>162</v>
       </c>
       <c r="H62">
-        <v>164.5</v>
+        <v>166.5</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>722</v>
+        <v>716</v>
       </c>
       <c r="B63" t="s">
-        <v>723</v>
+        <v>717</v>
       </c>
       <c r="C63">
-        <v>4556</v>
+        <v>2498</v>
       </c>
       <c r="D63">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E63" t="s">
         <v>10</v>
       </c>
       <c r="F63" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G63">
-        <v>900</v>
+        <v>92</v>
       </c>
       <c r="H63">
-        <v>927</v>
+        <v>94</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B64" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="C64">
-        <v>4557</v>
+        <v>2806</v>
       </c>
       <c r="D64">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E64" t="s">
         <v>10</v>
       </c>
       <c r="F64" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="G64">
-        <v>182</v>
+        <v>472.5</v>
       </c>
       <c r="H64">
-        <v>187.5</v>
+        <v>487</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
       <c r="B65" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
       <c r="C65">
-        <v>4018</v>
+        <v>2807</v>
       </c>
       <c r="D65">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E65" t="s">
         <v>10</v>
       </c>
       <c r="F65" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G65">
-        <v>230</v>
+        <v>159.5</v>
       </c>
       <c r="H65">
-        <v>240</v>
+        <v>164.5</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="B66" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="C66">
-        <v>2652</v>
+        <v>4556</v>
       </c>
       <c r="D66">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E66" t="s">
         <v>10</v>
       </c>
       <c r="F66" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G66">
-        <v>117</v>
+        <v>900</v>
       </c>
       <c r="H66">
-        <v>120.5</v>
+        <v>927</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
       <c r="B67" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
       <c r="C67">
-        <v>4049</v>
+        <v>4557</v>
       </c>
       <c r="D67">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E67" t="s">
         <v>10</v>
@@ -7306,24 +7318,24 @@
         <v>11</v>
       </c>
       <c r="G67">
-        <v>210</v>
+        <v>182</v>
       </c>
       <c r="H67">
-        <v>213.5</v>
+        <v>187.5</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="B68" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="C68">
-        <v>3737</v>
+        <v>4018</v>
       </c>
       <c r="D68">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E68" t="s">
         <v>10</v>
@@ -7332,24 +7344,24 @@
         <v>11</v>
       </c>
       <c r="G68">
-        <v>107</v>
+        <v>230</v>
       </c>
       <c r="H68">
-        <v>110</v>
+        <v>240</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="B69" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="C69">
-        <v>4301</v>
+        <v>2652</v>
       </c>
       <c r="D69">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E69" t="s">
         <v>10</v>
@@ -7358,24 +7370,24 @@
         <v>11</v>
       </c>
       <c r="G69">
-        <v>235</v>
+        <v>117</v>
       </c>
       <c r="H69">
-        <v>242</v>
+        <v>120.5</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="B70" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
       <c r="C70">
-        <v>4334</v>
+        <v>4049</v>
       </c>
       <c r="D70">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E70" t="s">
         <v>10</v>
@@ -7384,50 +7396,50 @@
         <v>11</v>
       </c>
       <c r="G70">
-        <v>376.5</v>
+        <v>210</v>
       </c>
       <c r="H70">
-        <v>388</v>
+        <v>213.5</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>89</v>
+        <v>726</v>
       </c>
       <c r="B71" t="s">
-        <v>90</v>
+        <v>727</v>
       </c>
       <c r="C71">
-        <v>195</v>
+        <v>3737</v>
       </c>
       <c r="D71">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E71" t="s">
         <v>10</v>
       </c>
       <c r="F71" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G71">
-        <v>255</v>
+        <v>107</v>
       </c>
       <c r="H71">
-        <v>262.5</v>
+        <v>110</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>89</v>
+        <v>728</v>
       </c>
       <c r="B72" t="s">
-        <v>90</v>
+        <v>729</v>
       </c>
       <c r="C72">
-        <v>54</v>
+        <v>4301</v>
       </c>
       <c r="D72">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E72" t="s">
         <v>10</v>
@@ -7436,128 +7448,128 @@
         <v>11</v>
       </c>
       <c r="G72">
-        <v>53</v>
+        <v>235</v>
       </c>
       <c r="H72">
-        <v>54.5</v>
+        <v>242</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="B73" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="C73">
-        <v>63</v>
+        <v>4334</v>
       </c>
       <c r="D73">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E73" t="s">
         <v>10</v>
       </c>
       <c r="F73" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G73">
-        <v>255</v>
+        <v>376.5</v>
       </c>
       <c r="H73">
-        <v>244.5</v>
+        <v>388</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>732</v>
+        <v>89</v>
       </c>
       <c r="B74" t="s">
-        <v>733</v>
+        <v>90</v>
       </c>
       <c r="C74">
-        <v>2483</v>
+        <v>195</v>
       </c>
       <c r="D74">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E74" t="s">
         <v>10</v>
       </c>
       <c r="F74" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G74">
-        <v>53</v>
+        <v>255</v>
       </c>
       <c r="H74">
-        <v>51</v>
+        <v>262.5</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>734</v>
+        <v>89</v>
       </c>
       <c r="B75" t="s">
-        <v>735</v>
+        <v>90</v>
       </c>
       <c r="C75">
-        <v>2974</v>
+        <v>54</v>
       </c>
       <c r="D75">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E75" t="s">
         <v>10</v>
       </c>
       <c r="F75" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G75">
-        <v>250</v>
+        <v>53</v>
       </c>
       <c r="H75">
-        <v>257.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="B76" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C76">
-        <v>2831</v>
+        <v>63</v>
       </c>
       <c r="D76">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E76" t="s">
         <v>10</v>
       </c>
       <c r="F76" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G76">
-        <v>127</v>
+        <v>255</v>
       </c>
       <c r="H76">
-        <v>131</v>
+        <v>244.5</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>736</v>
+        <v>732</v>
       </c>
       <c r="B77" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
       <c r="C77">
-        <v>4137</v>
+        <v>2483</v>
       </c>
       <c r="D77">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E77" t="s">
         <v>10</v>
@@ -7566,47 +7578,47 @@
         <v>11</v>
       </c>
       <c r="G77">
-        <v>270</v>
+        <v>53</v>
       </c>
       <c r="H77">
-        <v>278</v>
+        <v>51</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="B78" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="C78">
-        <v>4380</v>
+        <v>2974</v>
       </c>
       <c r="D78">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E78" t="s">
         <v>10</v>
       </c>
       <c r="F78" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G78">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="H78">
-        <v>278</v>
+        <v>257.5</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>740</v>
+        <v>734</v>
       </c>
       <c r="B79" t="s">
-        <v>741</v>
+        <v>735</v>
       </c>
       <c r="C79">
-        <v>4566</v>
+        <v>2831</v>
       </c>
       <c r="D79">
         <v>5</v>
@@ -7618,24 +7630,24 @@
         <v>11</v>
       </c>
       <c r="G79">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="H79">
-        <v>247</v>
+        <v>131</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>742</v>
+        <v>736</v>
       </c>
       <c r="B80" t="s">
-        <v>743</v>
+        <v>737</v>
       </c>
       <c r="C80">
-        <v>4567</v>
+        <v>4137</v>
       </c>
       <c r="D80">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E80" t="s">
         <v>10</v>
@@ -7644,24 +7656,24 @@
         <v>11</v>
       </c>
       <c r="G80">
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="H80">
-        <v>247</v>
+        <v>278</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>744</v>
+        <v>738</v>
       </c>
       <c r="B81" t="s">
-        <v>745</v>
+        <v>739</v>
       </c>
       <c r="C81">
-        <v>4204</v>
+        <v>4380</v>
       </c>
       <c r="D81">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E81" t="s">
         <v>10</v>
@@ -7670,50 +7682,50 @@
         <v>11</v>
       </c>
       <c r="G81">
-        <v>145.5</v>
+        <v>270</v>
       </c>
       <c r="H81">
-        <v>150</v>
+        <v>278</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
       <c r="B82" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="C82">
-        <v>4205</v>
+        <v>4566</v>
       </c>
       <c r="D82">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E82" t="s">
         <v>10</v>
       </c>
       <c r="F82" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G82">
-        <v>360</v>
+        <v>240</v>
       </c>
       <c r="H82">
-        <v>371</v>
+        <v>247</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="B83" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="C83">
-        <v>4225</v>
+        <v>4567</v>
       </c>
       <c r="D83">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E83" t="s">
         <v>10</v>
@@ -7722,50 +7734,50 @@
         <v>11</v>
       </c>
       <c r="G83">
-        <v>900</v>
+        <v>240</v>
       </c>
       <c r="H83">
-        <v>927</v>
+        <v>247</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="B84" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="C84">
-        <v>4378</v>
+        <v>4204</v>
       </c>
       <c r="D84">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E84" t="s">
         <v>10</v>
       </c>
       <c r="F84" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G84">
-        <v>430</v>
+        <v>145.5</v>
       </c>
       <c r="H84">
-        <v>443</v>
+        <v>150</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="B85" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="C85">
-        <v>4379</v>
+        <v>4205</v>
       </c>
       <c r="D85">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E85" t="s">
         <v>10</v>
@@ -7774,258 +7786,258 @@
         <v>14</v>
       </c>
       <c r="G85">
-        <v>43</v>
+        <v>360</v>
       </c>
       <c r="H85">
-        <v>44.5</v>
+        <v>371</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="B86" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="C86">
-        <v>3524</v>
+        <v>4225</v>
       </c>
       <c r="D86">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E86" t="s">
         <v>10</v>
       </c>
       <c r="F86" t="s">
-        <v>750</v>
+        <v>11</v>
       </c>
       <c r="G86">
-        <v>350</v>
+        <v>900</v>
       </c>
       <c r="H86">
-        <v>360.5</v>
+        <v>927</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="B87" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="C87">
-        <v>3523</v>
+        <v>4378</v>
       </c>
       <c r="D87">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E87" t="s">
         <v>10</v>
       </c>
       <c r="F87" t="s">
-        <v>750</v>
+        <v>14</v>
       </c>
       <c r="G87">
-        <v>72</v>
+        <v>430</v>
       </c>
       <c r="H87">
-        <v>74</v>
+        <v>443</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>751</v>
+        <v>746</v>
       </c>
       <c r="B88" t="s">
-        <v>752</v>
+        <v>747</v>
       </c>
       <c r="C88">
-        <v>3521</v>
+        <v>4379</v>
       </c>
       <c r="D88">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E88" t="s">
-        <v>753</v>
+        <v>10</v>
       </c>
       <c r="F88" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G88">
-        <v>158</v>
+        <v>43</v>
       </c>
       <c r="H88">
-        <v>163</v>
+        <v>44.5</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="B89" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="C89">
-        <v>3522</v>
+        <v>3524</v>
       </c>
       <c r="D89">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E89" t="s">
-        <v>408</v>
+        <v>10</v>
       </c>
       <c r="F89" t="s">
-        <v>25</v>
+        <v>750</v>
       </c>
       <c r="G89">
-        <v>216.5</v>
+        <v>350</v>
       </c>
       <c r="H89">
-        <v>223</v>
+        <v>360.5</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>754</v>
+        <v>748</v>
       </c>
       <c r="B90" t="s">
-        <v>755</v>
+        <v>749</v>
       </c>
       <c r="C90">
-        <v>64</v>
+        <v>3523</v>
       </c>
       <c r="D90">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E90" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F90" t="s">
-        <v>25</v>
+        <v>750</v>
       </c>
       <c r="G90">
-        <v>132</v>
+        <v>72</v>
       </c>
       <c r="H90">
-        <v>136</v>
+        <v>74</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>756</v>
+        <v>751</v>
       </c>
       <c r="B91" t="s">
-        <v>757</v>
+        <v>752</v>
       </c>
       <c r="C91">
-        <v>90</v>
+        <v>3521</v>
       </c>
       <c r="D91">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E91" t="s">
-        <v>30</v>
+        <v>753</v>
       </c>
       <c r="F91" t="s">
         <v>25</v>
       </c>
       <c r="G91">
-        <v>132</v>
+        <v>158</v>
       </c>
       <c r="H91">
-        <v>136</v>
+        <v>163</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>758</v>
+        <v>751</v>
       </c>
       <c r="B92" t="s">
-        <v>759</v>
+        <v>752</v>
       </c>
       <c r="C92">
-        <v>3637</v>
+        <v>3522</v>
       </c>
       <c r="D92">
+        <v>12</v>
+      </c>
+      <c r="E92" t="s">
+        <v>408</v>
+      </c>
+      <c r="F92" t="s">
         <v>25</v>
       </c>
-      <c r="E92" t="s">
-        <v>10</v>
-      </c>
-      <c r="F92" t="s">
-        <v>14</v>
-      </c>
       <c r="G92">
-        <v>375</v>
+        <v>216.5</v>
       </c>
       <c r="H92">
-        <v>386</v>
+        <v>223</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="B93" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="C93">
-        <v>2805</v>
+        <v>64</v>
       </c>
       <c r="D93">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E93" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F93" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G93">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="H93">
-        <v>154.5</v>
+        <v>136</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="B94" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="C94">
-        <v>2427</v>
+        <v>90</v>
       </c>
       <c r="D94">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E94" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F94" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G94">
-        <v>46</v>
+        <v>132</v>
       </c>
       <c r="H94">
-        <v>47.5</v>
+        <v>136</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="B95" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="C95">
-        <v>3437</v>
+        <v>3637</v>
       </c>
       <c r="D95">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E95" t="s">
         <v>10</v>
@@ -8034,284 +8046,284 @@
         <v>14</v>
       </c>
       <c r="G95">
-        <v>390</v>
+        <v>375</v>
       </c>
       <c r="H95">
-        <v>402</v>
+        <v>386</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="B96" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="C96">
-        <v>3396</v>
+        <v>2805</v>
       </c>
       <c r="D96">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E96" t="s">
         <v>10</v>
       </c>
       <c r="F96" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G96">
-        <v>197</v>
+        <v>150</v>
       </c>
       <c r="H96">
-        <v>203</v>
+        <v>154.5</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="B97" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="C97">
-        <v>3395</v>
+        <v>2427</v>
       </c>
       <c r="D97">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E97" t="s">
-        <v>764</v>
+        <v>10</v>
       </c>
       <c r="F97" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G97">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="H97">
-        <v>55.5</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>765</v>
+        <v>760</v>
       </c>
       <c r="B98" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
       <c r="C98">
-        <v>3490</v>
+        <v>3437</v>
       </c>
       <c r="D98">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E98" t="s">
-        <v>764</v>
+        <v>10</v>
       </c>
       <c r="F98" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G98">
-        <v>169</v>
+        <v>390</v>
       </c>
       <c r="H98">
-        <v>174</v>
+        <v>402</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>767</v>
+        <v>760</v>
       </c>
       <c r="B99" t="s">
-        <v>768</v>
+        <v>761</v>
       </c>
       <c r="C99">
-        <v>458</v>
+        <v>3396</v>
       </c>
       <c r="D99">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E99" t="s">
-        <v>769</v>
+        <v>10</v>
       </c>
       <c r="F99" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G99">
-        <v>269.5</v>
+        <v>197</v>
       </c>
       <c r="H99">
-        <v>278</v>
+        <v>203</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>770</v>
+        <v>762</v>
       </c>
       <c r="B100" t="s">
-        <v>771</v>
+        <v>763</v>
       </c>
       <c r="C100">
-        <v>2641</v>
+        <v>3395</v>
       </c>
       <c r="D100">
         <v>12</v>
       </c>
       <c r="E100" t="s">
-        <v>769</v>
+        <v>764</v>
       </c>
       <c r="F100" t="s">
         <v>25</v>
       </c>
       <c r="G100">
-        <v>222</v>
+        <v>54</v>
       </c>
       <c r="H100">
-        <v>229</v>
+        <v>55.5</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>772</v>
+        <v>765</v>
       </c>
       <c r="B101" t="s">
-        <v>773</v>
+        <v>766</v>
       </c>
       <c r="C101">
-        <v>4293</v>
+        <v>3490</v>
       </c>
       <c r="D101">
         <v>12</v>
       </c>
       <c r="E101" t="s">
-        <v>769</v>
+        <v>764</v>
       </c>
       <c r="F101" t="s">
         <v>25</v>
       </c>
       <c r="G101">
-        <v>210</v>
+        <v>169</v>
       </c>
       <c r="H101">
-        <v>216.5</v>
+        <v>174</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>774</v>
+        <v>767</v>
       </c>
       <c r="B102" t="s">
-        <v>775</v>
+        <v>768</v>
       </c>
       <c r="C102">
-        <v>2396</v>
+        <v>458</v>
       </c>
       <c r="D102">
+        <v>12</v>
+      </c>
+      <c r="E102" t="s">
+        <v>769</v>
+      </c>
+      <c r="F102" t="s">
         <v>25</v>
       </c>
-      <c r="E102" t="s">
-        <v>10</v>
-      </c>
-      <c r="F102" t="s">
-        <v>14</v>
-      </c>
       <c r="G102">
-        <v>675</v>
+        <v>269.5</v>
       </c>
       <c r="H102">
-        <v>695.5</v>
+        <v>278</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
       <c r="B103" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="C103">
-        <v>2426</v>
+        <v>2641</v>
       </c>
       <c r="D103">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E103" t="s">
-        <v>10</v>
+        <v>769</v>
       </c>
       <c r="F103" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G103">
-        <v>137</v>
+        <v>222</v>
       </c>
       <c r="H103">
-        <v>141</v>
+        <v>229</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="B104" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="C104">
-        <v>4335</v>
+        <v>4293</v>
       </c>
       <c r="D104">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E104" t="s">
-        <v>10</v>
+        <v>769</v>
       </c>
       <c r="F104" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G104">
-        <v>440</v>
+        <v>210</v>
       </c>
       <c r="H104">
-        <v>440</v>
+        <v>216.5</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="B105" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="C105">
-        <v>4477</v>
+        <v>2396</v>
       </c>
       <c r="D105">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="E105" t="s">
         <v>10</v>
       </c>
       <c r="F105" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G105">
-        <v>252</v>
+        <v>675</v>
       </c>
       <c r="H105">
-        <v>259.5</v>
+        <v>695.5</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>780</v>
+        <v>774</v>
       </c>
       <c r="B106" t="s">
-        <v>781</v>
+        <v>775</v>
       </c>
       <c r="C106">
-        <v>4479</v>
+        <v>2426</v>
       </c>
       <c r="D106">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E106" t="s">
         <v>10</v>
@@ -8320,21 +8332,21 @@
         <v>11</v>
       </c>
       <c r="G106">
-        <v>252</v>
+        <v>137</v>
       </c>
       <c r="H106">
-        <v>259.5</v>
+        <v>141</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>782</v>
+        <v>776</v>
       </c>
       <c r="B107" t="s">
-        <v>783</v>
+        <v>777</v>
       </c>
       <c r="C107">
-        <v>4478</v>
+        <v>4335</v>
       </c>
       <c r="D107">
         <v>3</v>
@@ -8346,165 +8358,243 @@
         <v>11</v>
       </c>
       <c r="G107">
-        <v>252</v>
+        <v>440</v>
       </c>
       <c r="H107">
-        <v>259.5</v>
+        <v>440</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>784</v>
+        <v>778</v>
       </c>
       <c r="B108" t="s">
-        <v>785</v>
+        <v>779</v>
       </c>
       <c r="C108">
-        <v>2646</v>
+        <v>4477</v>
       </c>
       <c r="D108">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E108" t="s">
-        <v>786</v>
+        <v>10</v>
       </c>
       <c r="F108" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="G108">
-        <v>50.5</v>
+        <v>252</v>
       </c>
       <c r="H108">
-        <v>52</v>
+        <v>259.5</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>784</v>
+        <v>780</v>
       </c>
       <c r="B109" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="C109">
-        <v>2645</v>
+        <v>4479</v>
       </c>
       <c r="D109">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E109" t="s">
-        <v>787</v>
+        <v>10</v>
       </c>
       <c r="F109" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="G109">
-        <v>78</v>
+        <v>252</v>
       </c>
       <c r="H109">
-        <v>80</v>
+        <v>259.5</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="B110" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="C110">
-        <v>2638</v>
+        <v>4478</v>
       </c>
       <c r="D110">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E110" t="s">
-        <v>788</v>
+        <v>10</v>
       </c>
       <c r="F110" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="G110">
-        <v>65</v>
+        <v>252</v>
       </c>
       <c r="H110">
-        <v>67</v>
+        <v>259.5</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
       <c r="B111" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="C111">
-        <v>4294</v>
+        <v>2646</v>
       </c>
       <c r="D111">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E111" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
       <c r="F111" t="s">
         <v>33</v>
       </c>
       <c r="G111">
-        <v>150</v>
+        <v>53</v>
       </c>
       <c r="H111">
-        <v>154.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>792</v>
+        <v>784</v>
       </c>
       <c r="B112" t="s">
-        <v>793</v>
+        <v>785</v>
       </c>
       <c r="C112">
-        <v>4314</v>
+        <v>2645</v>
       </c>
       <c r="D112">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E112" t="s">
-        <v>408</v>
+        <v>787</v>
       </c>
       <c r="F112" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G112">
-        <v>252</v>
+        <v>81.5</v>
       </c>
       <c r="H112">
-        <v>260</v>
+        <v>84</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
+        <v>784</v>
+      </c>
+      <c r="B113" t="s">
+        <v>785</v>
+      </c>
+      <c r="C113">
+        <v>2638</v>
+      </c>
+      <c r="D113">
+        <v>9</v>
+      </c>
+      <c r="E113" t="s">
+        <v>788</v>
+      </c>
+      <c r="F113" t="s">
+        <v>33</v>
+      </c>
+      <c r="G113">
+        <v>70</v>
+      </c>
+      <c r="H113">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>789</v>
+      </c>
+      <c r="B114" t="s">
+        <v>790</v>
+      </c>
+      <c r="C114">
+        <v>4294</v>
+      </c>
+      <c r="D114">
+        <v>18</v>
+      </c>
+      <c r="E114" t="s">
+        <v>791</v>
+      </c>
+      <c r="F114" t="s">
+        <v>33</v>
+      </c>
+      <c r="G114">
+        <v>150</v>
+      </c>
+      <c r="H114">
+        <v>154.5</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>792</v>
+      </c>
+      <c r="B115" t="s">
+        <v>793</v>
+      </c>
+      <c r="C115">
+        <v>4314</v>
+      </c>
+      <c r="D115">
+        <v>15</v>
+      </c>
+      <c r="E115" t="s">
+        <v>408</v>
+      </c>
+      <c r="F115" t="s">
+        <v>25</v>
+      </c>
+      <c r="G115">
+        <v>252</v>
+      </c>
+      <c r="H115">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
         <v>794</v>
       </c>
-      <c r="B113" t="s">
+      <c r="B116" t="s">
         <v>795</v>
       </c>
-      <c r="C113">
+      <c r="C116">
         <v>4315</v>
       </c>
-      <c r="D113">
+      <c r="D116">
         <v>15</v>
       </c>
-      <c r="E113" t="s">
+      <c r="E116" t="s">
         <v>796</v>
       </c>
-      <c r="F113" t="s">
+      <c r="F116" t="s">
         <v>25</v>
       </c>
-      <c r="G113">
+      <c r="G116">
         <v>450</v>
       </c>
-      <c r="H113">
+      <c r="H116">
         <v>463.5</v>
       </c>
     </row>
@@ -13038,10 +13128,10 @@
         <v>33</v>
       </c>
       <c r="G120">
-        <v>27.5</v>
+        <v>30</v>
       </c>
       <c r="H120">
-        <v>28.5</v>
+        <v>31</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.25">
@@ -13064,10 +13154,10 @@
         <v>33</v>
       </c>
       <c r="G121">
-        <v>24.5</v>
+        <v>25.5</v>
       </c>
       <c r="H121">
-        <v>25</v>
+        <v>26.5</v>
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Atualizando preço e mais uma mercadoria 21/05
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodosLibanes.xlsx
+++ b/data/ProdutosFomatodosLibanes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\listaProdutosToufic\lista-de-produtos-toufic\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDA5D795-263B-421C-8C22-3DE2DDAB0DCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C155E12B-6BF2-41A5-ACE3-5C29FA7E6C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" firstSheet="11" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3592" uniqueCount="1111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3596" uniqueCount="1114">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -3370,6 +3370,15 @@
   </si>
   <si>
     <t>FLOCOS DE ARROZ</t>
+  </si>
+  <si>
+    <t>pacoca-de-amendoim-espeto</t>
+  </si>
+  <si>
+    <t>PAÇOCA DE AMENDOIM ESPETO</t>
+  </si>
+  <si>
+    <t>X90G</t>
   </si>
 </sst>
 </file>
@@ -10003,7 +10012,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
-  <dimension ref="A1:H122"/>
+  <dimension ref="A1:H123"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -12660,10 +12669,10 @@
         <v>988</v>
       </c>
       <c r="G102">
-        <v>71.5</v>
+        <v>75.5</v>
       </c>
       <c r="H102">
-        <v>73.5</v>
+        <v>78</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
@@ -13032,65 +13041,65 @@
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>1051</v>
+        <v>1111</v>
       </c>
       <c r="B117" t="s">
-        <v>1052</v>
+        <v>1112</v>
       </c>
       <c r="C117">
-        <v>4123</v>
+        <v>4582</v>
       </c>
       <c r="D117">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E117" t="s">
-        <v>1016</v>
+        <v>1113</v>
       </c>
       <c r="F117" t="s">
         <v>11</v>
       </c>
       <c r="G117">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="H117">
-        <v>62</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="B118" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="C118">
-        <v>4306</v>
+        <v>4123</v>
       </c>
       <c r="D118">
         <v>10</v>
       </c>
       <c r="E118" t="s">
-        <v>1003</v>
+        <v>1016</v>
       </c>
       <c r="F118" t="s">
-        <v>988</v>
+        <v>11</v>
       </c>
       <c r="G118">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="H118">
-        <v>83.5</v>
+        <v>62</v>
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
       <c r="B119" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="C119">
-        <v>4307</v>
+        <v>4306</v>
       </c>
       <c r="D119">
         <v>10</v>
@@ -13110,28 +13119,28 @@
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="B120" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C120">
-        <v>2659</v>
+        <v>4307</v>
       </c>
       <c r="D120">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E120" t="s">
-        <v>1059</v>
+        <v>1003</v>
       </c>
       <c r="F120" t="s">
-        <v>33</v>
+        <v>988</v>
       </c>
       <c r="G120">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="H120">
-        <v>31</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.25">
@@ -13142,47 +13151,73 @@
         <v>1058</v>
       </c>
       <c r="C121">
-        <v>2621</v>
+        <v>2659</v>
       </c>
       <c r="D121">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E121" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="F121" t="s">
         <v>33</v>
       </c>
       <c r="G121">
-        <v>25.5</v>
+        <v>30</v>
       </c>
       <c r="H121">
-        <v>26.5</v>
+        <v>31</v>
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>1061</v>
+        <v>1057</v>
       </c>
       <c r="B122" t="s">
-        <v>1062</v>
+        <v>1058</v>
       </c>
       <c r="C122">
-        <v>3656</v>
+        <v>2621</v>
       </c>
       <c r="D122">
         <v>5</v>
       </c>
       <c r="E122" t="s">
-        <v>1003</v>
+        <v>1060</v>
       </c>
       <c r="F122" t="s">
         <v>33</v>
       </c>
       <c r="G122">
+        <v>25.5</v>
+      </c>
+      <c r="H122">
+        <v>26.5</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B123" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C123">
+        <v>3656</v>
+      </c>
+      <c r="D123">
+        <v>5</v>
+      </c>
+      <c r="E123" t="s">
+        <v>1003</v>
+      </c>
+      <c r="F123" t="s">
+        <v>33</v>
+      </c>
+      <c r="G123">
         <v>27</v>
       </c>
-      <c r="H122">
+      <c r="H123">
         <v>28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizando o preço 25/05
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodosLibanes.xlsx
+++ b/data/ProdutosFomatodosLibanes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\listaProdutosToufic\lista-de-produtos-toufic\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61851D42-DD5D-450F-BC7A-C1FB74E96172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB1A7A38-A70D-46CF-B802-B0501E06D81D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="345" yWindow="945" windowWidth="27300" windowHeight="13920" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="promoçoes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3612" uniqueCount="1117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3608" uniqueCount="1117">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -3740,7 +3740,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
@@ -3780,39 +3780,39 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C2">
-        <v>2229</v>
+        <v>195</v>
       </c>
       <c r="D2">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G2">
-        <v>145</v>
+        <v>245</v>
       </c>
       <c r="H2">
-        <v>180</v>
+        <v>262.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C3">
-        <v>195</v>
+        <v>569</v>
       </c>
       <c r="D3">
         <v>25</v>
@@ -3824,21 +3824,21 @@
         <v>14</v>
       </c>
       <c r="G3">
-        <v>245</v>
+        <v>117</v>
       </c>
       <c r="H3">
-        <v>262.5</v>
+        <v>121.5</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C4">
-        <v>569</v>
+        <v>282</v>
       </c>
       <c r="D4">
         <v>25</v>
@@ -3858,13 +3858,13 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>93</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
+        <v>35</v>
       </c>
       <c r="C5">
-        <v>282</v>
+        <v>564</v>
       </c>
       <c r="D5">
         <v>25</v>
@@ -3884,13 +3884,13 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>95</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>96</v>
       </c>
       <c r="C6">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D6">
         <v>25</v>
@@ -3902,21 +3902,21 @@
         <v>14</v>
       </c>
       <c r="G6">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="H6">
-        <v>121.5</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C7">
-        <v>565</v>
+        <v>109</v>
       </c>
       <c r="D7">
         <v>25</v>
@@ -3928,21 +3928,21 @@
         <v>14</v>
       </c>
       <c r="G7">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="H7">
-        <v>129</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C8">
-        <v>109</v>
+        <v>3110</v>
       </c>
       <c r="D8">
         <v>25</v>
@@ -3954,21 +3954,21 @@
         <v>14</v>
       </c>
       <c r="G8">
-        <v>155</v>
+        <v>81</v>
       </c>
       <c r="H8">
-        <v>162</v>
+        <v>91.5</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C9">
-        <v>3110</v>
+        <v>8</v>
       </c>
       <c r="D9">
         <v>25</v>
@@ -3980,35 +3980,9 @@
         <v>14</v>
       </c>
       <c r="G9">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H9">
-        <v>91.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>101</v>
-      </c>
-      <c r="B10" t="s">
-        <v>102</v>
-      </c>
-      <c r="C10">
-        <v>8</v>
-      </c>
-      <c r="D10">
-        <v>25</v>
-      </c>
-      <c r="E10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10">
-        <v>88</v>
-      </c>
-      <c r="H10">
         <v>94</v>
       </c>
     </row>
@@ -4622,7 +4596,7 @@
         <v>25</v>
       </c>
       <c r="G23">
-        <v>140</v>
+        <v>175</v>
       </c>
       <c r="H23">
         <v>180</v>

</xml_diff>